<commit_message>
feat: template import transaksi berformat Excel rapi
- Buat scripts/generate-import-template.ts: generator template Excel
  dengan 2 sheet (Data Import + Panduan), 18 kolom, 3 baris contoh
- Regenerate public/templates/mobeng-transaction-import-template.xlsx
  dengan header berlabel Indonesia, keterangan wajib/opsional, contoh nilai
- Update link download di transaction-import-panel dari CSV ke XLSX
- Tambah script npm gen:template untuk regenerasi template
</commit_message>
<xml_diff>
--- a/public/templates/mobeng-transaction-import-template.xlsx
+++ b/public/templates/mobeng-transaction-import-template.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="transactions" sheetId="1" r:id="rId1"/>
+    <sheet name="Data Import" sheetId="1" r:id="rId1"/>
+    <sheet name="Panduan" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,123 +398,693 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R9"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+    <col min="13" max="13" width="38.83203125" customWidth="1"/>
+    <col min="14" max="14" width="34.83203125" customWidth="1"/>
+    <col min="15" max="15" width="22.83203125" customWidth="1"/>
+    <col min="16" max="16" width="24.83203125" customWidth="1"/>
+    <col min="17" max="17" width="24.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>invoice_number</v>
+        <v>No. Invoice</v>
       </c>
       <c r="B1" t="str">
-        <v>transaction_date</v>
+        <v>Tgl. Transaksi</v>
       </c>
       <c r="C1" t="str">
-        <v>branch_name</v>
+        <v>Nama Cabang</v>
       </c>
       <c r="D1" t="str">
-        <v>customer_name</v>
+        <v>Nama Pelanggan</v>
       </c>
       <c r="E1" t="str">
-        <v>customer_phone</v>
+        <v>No. HP Pelanggan</v>
       </c>
       <c r="F1" t="str">
-        <v>customer_email</v>
+        <v>Email Pelanggan</v>
       </c>
       <c r="G1" t="str">
-        <v>vehicle_plate</v>
+        <v>Plat Nomor</v>
       </c>
       <c r="H1" t="str">
-        <v>vehicle_brand</v>
+        <v>Merek Kendaraan</v>
       </c>
       <c r="I1" t="str">
-        <v>vehicle_model</v>
+        <v>Model Kendaraan</v>
       </c>
       <c r="J1" t="str">
-        <v>vehicle_year</v>
+        <v>Tahun Kendaraan</v>
       </c>
       <c r="K1" t="str">
-        <v>mileage</v>
+        <v>Odometer (km)</v>
       </c>
       <c r="L1" t="str">
-        <v>service_category</v>
+        <v>Kategori Servis</v>
       </c>
       <c r="M1" t="str">
-        <v>service_description</v>
+        <v>Deskripsi Servis</v>
       </c>
       <c r="N1" t="str">
-        <v>parts_replaced</v>
+        <v>Sparepart Diganti</v>
       </c>
       <c r="O1" t="str">
-        <v>total_amount</v>
+        <v>Total Tagihan (Rp)</v>
       </c>
       <c r="P1" t="str">
-        <v>service_advisor</v>
+        <v>Service Advisor</v>
       </c>
       <c r="Q1" t="str">
-        <v>technician_name</v>
+        <v>Nama Teknisi</v>
       </c>
       <c r="R1" t="str">
-        <v>payment_status</v>
+        <v>Status Pembayaran</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>INV-MBG-0001</v>
+        <v>invoice_number</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-10T10:30:00+07:00</v>
+        <v>transaction_date</v>
       </c>
       <c r="C2" t="str">
-        <v>Mobeng BSD</v>
+        <v>branch_name</v>
       </c>
       <c r="D2" t="str">
-        <v>Andi Pratama</v>
+        <v>customer_name</v>
       </c>
       <c r="E2" t="str">
-        <v>081234567890</v>
+        <v>customer_phone</v>
       </c>
       <c r="F2" t="str">
-        <v>andi@example.com</v>
+        <v>customer_email</v>
       </c>
       <c r="G2" t="str">
-        <v>B1234XYZ</v>
+        <v>vehicle_plate</v>
       </c>
       <c r="H2" t="str">
+        <v>vehicle_brand</v>
+      </c>
+      <c r="I2" t="str">
+        <v>vehicle_model</v>
+      </c>
+      <c r="J2" t="str">
+        <v>vehicle_year</v>
+      </c>
+      <c r="K2" t="str">
+        <v>mileage</v>
+      </c>
+      <c r="L2" t="str">
+        <v>service_category</v>
+      </c>
+      <c r="M2" t="str">
+        <v>service_description</v>
+      </c>
+      <c r="N2" t="str">
+        <v>parts_replaced</v>
+      </c>
+      <c r="O2" t="str">
+        <v>total_amount</v>
+      </c>
+      <c r="P2" t="str">
+        <v>service_advisor</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>technician_name</v>
+      </c>
+      <c r="R2" t="str">
+        <v>payment_status</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="B3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="C3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="D3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="E3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="G3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="H3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="I3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="J3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="K3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="L3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="M3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="O3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="P3" t="str">
+        <v>WAJIB</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="R3" t="str">
+        <v>WAJIB</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Nomor invoice unik dari sistem bengkel</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Format: YYYY-MM-DD</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Harus sama persis dengan nama cabang di CRM</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Nama lengkap pelanggan</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Format tanpa tanda hubung atau spasi</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Plat nomor kendaraan</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Merek kendaraan</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Model/tipe kendaraan</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Tahun produksi (4 digit)</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Odometer saat masuk servis (angka)</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Contoh: Servis Berkala, Ganti Oli, Tune Up</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Detail pekerjaan yang dilakukan</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Nama sparepart yang diganti, opsional</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Nominal tagihan tanpa titik/koma (angka)</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Nama service advisor yang menangani</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Nama teknisi, opsional</v>
+      </c>
+      <c r="R4" t="str">
+        <v>PAID atau UNPAID</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>INV-2026-001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-05-10</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Mobeng Ciledug</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Budi Santoso</v>
+      </c>
+      <c r="E5" t="str">
+        <v>08121234567</v>
+      </c>
+      <c r="F5" t="str">
+        <v>budi@email.com</v>
+      </c>
+      <c r="G5" t="str">
+        <v>B 1234 XYZ</v>
+      </c>
+      <c r="H5" t="str">
         <v>Toyota</v>
       </c>
-      <c r="I2" t="str">
+      <c r="I5" t="str">
         <v>Avanza</v>
       </c>
-      <c r="J2">
+      <c r="J5" t="str">
+        <v>2021</v>
+      </c>
+      <c r="K5" t="str">
+        <v>45000</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Servis Berkala</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Ganti oli + filter oli</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Oli Shell Helix 5W-30</v>
+      </c>
+      <c r="O5" t="str">
+        <v>350000</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Andi Prasetyo</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Riko Wijaya</v>
+      </c>
+      <c r="R5" t="str">
+        <v>PAID</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>INV-2026-001</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-05-10</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Mobeng Ciledug</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Budi Santoso</v>
+      </c>
+      <c r="E7" t="str">
+        <v>08121234567</v>
+      </c>
+      <c r="F7" t="str">
+        <v>budi@email.com</v>
+      </c>
+      <c r="G7" t="str">
+        <v>B 1234 XYZ</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Toyota</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Avanza</v>
+      </c>
+      <c r="J7" t="str">
+        <v>2021</v>
+      </c>
+      <c r="K7" t="str">
+        <v>45000</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Servis Berkala</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Ganti oli + filter oli</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Oli Shell Helix 5W-30</v>
+      </c>
+      <c r="O7" t="str">
+        <v>350000</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Andi Prasetyo</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>Riko Wijaya</v>
+      </c>
+      <c r="R7" t="str">
+        <v>PAID</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>INV-2026-002</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-05-11</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Mobeng Ciledug</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Siti Rahayu</v>
+      </c>
+      <c r="E8" t="str">
+        <v>08567891234</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>B 9876 ABC</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Honda</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Jazz</v>
+      </c>
+      <c r="J8" t="str">
+        <v>2019</v>
+      </c>
+      <c r="K8" t="str">
+        <v>62000</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Tune Up</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Tune up + ganti busi</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Busi NGK x4</v>
+      </c>
+      <c r="O8" t="str">
+        <v>480000</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Dewi Lestari</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Agus Supriyanto</v>
+      </c>
+      <c r="R8" t="str">
+        <v>PAID</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>INV-2026-003</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-05-12</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Mobeng Tangerang</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Hendra Gunawan</v>
+      </c>
+      <c r="E9" t="str">
+        <v>08211112222</v>
+      </c>
+      <c r="F9" t="str">
+        <v>hendra@gmail.com</v>
+      </c>
+      <c r="G9" t="str">
+        <v>B 5555 DEF</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Daihatsu</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Xenia</v>
+      </c>
+      <c r="J9" t="str">
         <v>2020</v>
       </c>
-      <c r="K2">
-        <v>45210</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Oli Mobil</v>
-      </c>
-      <c r="M2" t="str">
-        <v>Ganti oli mesin + cek filter</v>
-      </c>
-      <c r="N2" t="str">
-        <v>Filter Oli,Engine Oil</v>
-      </c>
-      <c r="O2">
-        <v>850000</v>
-      </c>
-      <c r="P2" t="str">
-        <v>Ayu Lestari</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>Dimas Wijaya</v>
-      </c>
-      <c r="R2" t="str">
-        <v>PAID</v>
+      <c r="K9" t="str">
+        <v>38000</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Ganti Oli</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Ganti oli mesin saja</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Oli Pertamina Fastron 10W-40</v>
+      </c>
+      <c r="O9" t="str">
+        <v>220000</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Budi Hartono</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v>UNPAID</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A40"/>
+  <cols>
+    <col min="1" max="1" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PANDUAN IMPORT TRANSAKSI - MOBENG CRM</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>CARA PENGGUNAAN:</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>1. Isi data pada sheet 'Data Import' mulai dari baris ke-7 (baris data contoh bisa dihapus).</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2. Baris 1 (label), baris 2 (key), baris 3 (wajib/opsional), baris 4 (keterangan), baris 5 (contoh) JANGAN dihapus.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>3. Simpan file dalam format .xlsx atau .csv sebelum diupload.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>4. Maksimal 1000 baris data per upload.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>KETENTUAN KOLOM WAJIB:</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v xml:space="preserve">  • No. Invoice (invoice_number): Nomor invoice unik dari sistem bengkel</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v xml:space="preserve">  • Tgl. Transaksi (transaction_date): Format: YYYY-MM-DD</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v xml:space="preserve">  • Nama Cabang (branch_name): Harus sama persis dengan nama cabang di CRM</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v xml:space="preserve">  • Nama Pelanggan (customer_name): Nama lengkap pelanggan</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v xml:space="preserve">  • No. HP Pelanggan (customer_phone): Format tanpa tanda hubung atau spasi</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v xml:space="preserve">  • Plat Nomor (vehicle_plate): Plat nomor kendaraan</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v xml:space="preserve">  • Merek Kendaraan (vehicle_brand): Merek kendaraan</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v xml:space="preserve">  • Model Kendaraan (vehicle_model): Model/tipe kendaraan</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v xml:space="preserve">  • Tahun Kendaraan (vehicle_year): Tahun produksi (4 digit)</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v xml:space="preserve">  • Odometer (km) (mileage): Odometer saat masuk servis (angka)</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v xml:space="preserve">  • Kategori Servis (service_category): Contoh: Servis Berkala, Ganti Oli, Tune Up</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v xml:space="preserve">  • Deskripsi Servis (service_description): Detail pekerjaan yang dilakukan</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v xml:space="preserve">  • Total Tagihan (Rp) (total_amount): Nominal tagihan tanpa titik/koma (angka)</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v xml:space="preserve">  • Service Advisor (service_advisor): Nama service advisor yang menangani</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v xml:space="preserve">  • Status Pembayaran (payment_status): PAID atau UNPAID</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>KETENTUAN KOLOM OPSIONAL:</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v xml:space="preserve">  • Email Pelanggan (customer_email): Opsional</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v xml:space="preserve">  • Sparepart Diganti (parts_replaced): Nama sparepart yang diganti, opsional</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v xml:space="preserve">  • Nama Teknisi (technician_name): Nama teknisi, opsional</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>FORMAT NILAI:</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v xml:space="preserve">  • transaction_date: YYYY-MM-DD (contoh: 2026-05-10)</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v xml:space="preserve">  • total_amount: angka bulat tanpa titik/koma (contoh: 350000)</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v xml:space="preserve">  • mileage: angka bulat dalam km (contoh: 45000)</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v xml:space="preserve">  • vehicle_year: 4 digit tahun (contoh: 2021)</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v xml:space="preserve">  • payment_status: PAID atau UNPAID (huruf kapital)</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>CATATAN:</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v xml:space="preserve">  • Nama cabang (branch_name) harus sama persis dengan data cabang yang sudah terdaftar di CRM.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v xml:space="preserve">  • Nomor invoice harus unik. Duplikat akan di-skip atau di-update tergantung pilihan mode import.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>